<commit_message>
fix toolkit maturity scoring scale
</commit_message>
<xml_diff>
--- a/source/latest/AIMA_Assessment_Toolkit.xlsx
+++ b/source/latest/AIMA_Assessment_Toolkit.xlsx
@@ -86,13 +86,32 @@
     <t xml:space="preserve">Contributors:        The AIMA project team                                                                                                                                                                                        </t>
   </si>
   <si>
-    <t>Version: RC1</t>
+    <t>Version: 1.0.1</t>
   </si>
   <si>
     <t>OWASP AI Maturity Assessment (AIMA) Questions</t>
   </si>
   <si>
-    <t>Instructions: Answer each question with 0 (meaning no maturity) 0,33 (initial maturity), 0,66 (not full maturity) 1 (maturity). The maturity level for each practice area will be calculated based on your answers.</t>
+    <r>
+      <rPr>
+        <rFont val="Roboto Condensed"/>
+        <b/>
+        <i/>
+        <color rgb="FFFF0000"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t xml:space="preserve">Instructions: </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Roboto Condensed"/>
+        <b/>
+        <i/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t>Answer each question with 0 (meaning no maturity) 1 (initial maturity), 2 (not full maturity) 3 (maturity). The maturity level for each practice area will be calculated based on your answers.</t>
+    </r>
   </si>
   <si>
     <t>PRACTICE AREA</t>
@@ -892,11 +911,12 @@
     </font>
     <font>
       <b/>
-      <sz val="15.0"/>
+      <sz val="16.0"/>
       <color theme="1"/>
       <name val="Roboto Condensed"/>
     </font>
     <font>
+      <b/>
       <i/>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -921,7 +941,7 @@
     </font>
     <font>
       <b/>
-      <sz val="16.0"/>
+      <sz val="15.0"/>
       <color theme="1"/>
       <name val="Roboto Condensed"/>
     </font>
@@ -1454,7 +1474,7 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="15" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -1526,13 +1546,13 @@
     <xf borderId="9" fillId="0" fontId="11" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="7" fillId="13" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="7" fillId="13" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="10" fillId="0" fontId="11" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="7" fillId="13" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="7" fillId="13" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="11" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1541,7 +1561,7 @@
     <xf borderId="12" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="11" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="11" fillId="6" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="13" fillId="14" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -1550,10 +1570,10 @@
     <xf borderId="14" fillId="14" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="13" fillId="14" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="13" fillId="14" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="13" fillId="14" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="13" fillId="14" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="15" fillId="15" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -1562,49 +1582,49 @@
     <xf borderId="16" fillId="15" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="15" fillId="15" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="15" fillId="15" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="15" fillId="15" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="15" fillId="15" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="17" fillId="16" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="17" fillId="16" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="18" fillId="16" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="17" fillId="16" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="17" fillId="16" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="19" fillId="10" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="19" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="20" fillId="10" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="19" fillId="10" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="19" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="21" fillId="11" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="21" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="22" fillId="11" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="21" fillId="11" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="21" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="23" fillId="17" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="23" fillId="17" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="24" fillId="17" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="23" fillId="17" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="23" fillId="17" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="25" fillId="17" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="25" fillId="17" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="26" fillId="17" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1749,11 +1769,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1730178886"/>
-        <c:axId val="1055365087"/>
+        <c:axId val="608363380"/>
+        <c:axId val="1883651309"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1730178886"/>
+        <c:axId val="608363380"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1805,10 +1825,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1055365087"/>
+        <c:crossAx val="1883651309"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1055365087"/>
+        <c:axId val="1883651309"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1883,7 +1903,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1730178886"/>
+        <c:crossAx val="608363380"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -3518,7 +3538,7 @@
         <v>22</v>
       </c>
       <c r="F7" s="27">
-        <f>SUM(E7:E12)/2</f>
+        <f>SUM(E7:E12)/6</f>
         <v>0</v>
       </c>
       <c r="G7" s="12"/>
@@ -3749,7 +3769,7 @@
         <v>22</v>
       </c>
       <c r="F14" s="27">
-        <f>SUM(E14:E19)/2</f>
+        <f>SUM(E14:E19)/6</f>
         <v>0</v>
       </c>
       <c r="G14" s="12"/>
@@ -3980,7 +4000,7 @@
         <v>22</v>
       </c>
       <c r="F21" s="27">
-        <f>SUM(E21:E26)/2</f>
+        <f>SUM(E21:E26)/6</f>
         <v>0</v>
       </c>
       <c r="G21" s="12"/>
@@ -4236,7 +4256,7 @@
         <v>22</v>
       </c>
       <c r="F29" s="27">
-        <f>SUM(E29:E34)/2</f>
+        <f>SUM(E29:E34)/6</f>
         <v>0</v>
       </c>
       <c r="G29" s="12"/>
@@ -4467,7 +4487,7 @@
         <v>22</v>
       </c>
       <c r="F36" s="27">
-        <f>SUM(E36:E41)/2</f>
+        <f>SUM(E36:E41)/6</f>
         <v>0</v>
       </c>
       <c r="G36" s="12"/>
@@ -4698,7 +4718,7 @@
         <v>22</v>
       </c>
       <c r="F43" s="27">
-        <f>SUM(E43:E48)/2</f>
+        <f>SUM(E43:E48)/6</f>
         <v>0</v>
       </c>
       <c r="G43" s="12"/>
@@ -4954,7 +4974,7 @@
         <v>22</v>
       </c>
       <c r="F51" s="27">
-        <f>SUM(E51:E56)/2</f>
+        <f>SUM(E51:E56)/6</f>
         <v>0</v>
       </c>
       <c r="G51" s="12"/>
@@ -5185,7 +5205,7 @@
         <v>22</v>
       </c>
       <c r="F58" s="27">
-        <f>SUM(E58:E63)/2</f>
+        <f>SUM(E58:E63)/6</f>
         <v>0</v>
       </c>
       <c r="G58" s="12"/>
@@ -5416,7 +5436,7 @@
         <v>22</v>
       </c>
       <c r="F65" s="27">
-        <f>SUM(E65:E70)/2</f>
+        <f>SUM(E65:E70)/6</f>
         <v>0</v>
       </c>
       <c r="G65" s="12"/>
@@ -5672,7 +5692,7 @@
         <v>22</v>
       </c>
       <c r="F73" s="27">
-        <f>SUM(E73:E78)/2</f>
+        <f>SUM(E73:E78)/6</f>
         <v>0</v>
       </c>
       <c r="G73" s="12"/>
@@ -5903,7 +5923,7 @@
         <v>22</v>
       </c>
       <c r="F80" s="27">
-        <f>SUM(E80:E85)/2</f>
+        <f>SUM(E80:E85)/6</f>
         <v>0</v>
       </c>
       <c r="G80" s="12"/>
@@ -6134,7 +6154,7 @@
         <v>22</v>
       </c>
       <c r="F87" s="27">
-        <f>SUM(E87:E92)/2</f>
+        <f>SUM(E87:E92)/6</f>
         <v>0</v>
       </c>
       <c r="G87" s="12"/>
@@ -6390,7 +6410,7 @@
         <v>22</v>
       </c>
       <c r="F95" s="27">
-        <f>SUM(E95:E100)/2</f>
+        <f>SUM(E95:E100)/6</f>
         <v>0</v>
       </c>
       <c r="G95" s="12"/>
@@ -6621,7 +6641,7 @@
         <v>22</v>
       </c>
       <c r="F102" s="27">
-        <f>SUM(E102:E107)/2</f>
+        <f>SUM(E102:E107)/6</f>
         <v>0</v>
       </c>
       <c r="G102" s="12"/>
@@ -6852,7 +6872,7 @@
         <v>22</v>
       </c>
       <c r="F109" s="27">
-        <f>SUM(E109:E114)/2</f>
+        <f>SUM(E109:E114)/6</f>
         <v>0</v>
       </c>
       <c r="G109" s="12"/>
@@ -7108,7 +7128,7 @@
         <v>22</v>
       </c>
       <c r="F117" s="27">
-        <f>SUM(E117:E122)/2</f>
+        <f>SUM(E117:E122)/6</f>
         <v>0</v>
       </c>
       <c r="G117" s="12"/>
@@ -7339,7 +7359,7 @@
         <v>22</v>
       </c>
       <c r="F124" s="27">
-        <f>SUM(E124:E129)/2</f>
+        <f>SUM(E124:E129)/6</f>
         <v>0</v>
       </c>
       <c r="G124" s="12"/>
@@ -7570,7 +7590,7 @@
         <v>22</v>
       </c>
       <c r="F131" s="27">
-        <f>SUM(E131:E136)/2</f>
+        <f>SUM(E131:E136)/6</f>
         <v>0</v>
       </c>
       <c r="G131" s="12"/>
@@ -7826,7 +7846,7 @@
         <v>22</v>
       </c>
       <c r="F139" s="27">
-        <f>SUM(E139:E144)/2</f>
+        <f>SUM(E139:E144)/6</f>
         <v>0</v>
       </c>
       <c r="G139" s="12"/>
@@ -8057,7 +8077,7 @@
         <v>22</v>
       </c>
       <c r="F146" s="27">
-        <f>SUM(E146:E151)/2</f>
+        <f>SUM(E146:E151)/6</f>
         <v>0</v>
       </c>
       <c r="G146" s="12"/>
@@ -8288,7 +8308,7 @@
         <v>22</v>
       </c>
       <c r="F153" s="27">
-        <f>SUM(E153:E158)/2</f>
+        <f>SUM(E153:E158)/6</f>
         <v>0</v>
       </c>
       <c r="G153" s="12"/>
@@ -8544,7 +8564,7 @@
         <v>22</v>
       </c>
       <c r="F161" s="27">
-        <f>SUM(E161:E166)/2</f>
+        <f>SUM(E161:E166)/6</f>
         <v>0</v>
       </c>
       <c r="G161" s="12"/>
@@ -8775,7 +8795,7 @@
         <v>22</v>
       </c>
       <c r="F168" s="27">
-        <f>SUM(E168:E173)/2</f>
+        <f>SUM(E168:E173)/6</f>
         <v>0</v>
       </c>
       <c r="G168" s="12"/>
@@ -9006,7 +9026,7 @@
         <v>22</v>
       </c>
       <c r="F175" s="27">
-        <f>SUM(E175:E180)/2</f>
+        <f>SUM(E175:E180)/6</f>
         <v>0</v>
       </c>
       <c r="G175" s="12"/>
@@ -33112,23 +33132,24 @@
     <mergeCell ref="B167:H167"/>
     <mergeCell ref="B174:H174"/>
     <mergeCell ref="A181:H181"/>
-    <mergeCell ref="B28:H28"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="B6:H6"/>
     <mergeCell ref="F14:F19"/>
-    <mergeCell ref="F21:F26"/>
     <mergeCell ref="B20:H20"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="A7:A26"/>
+    <mergeCell ref="F7:F12"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="F36:F41"/>
+    <mergeCell ref="F43:F48"/>
+    <mergeCell ref="F21:F26"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="B28:H28"/>
+    <mergeCell ref="A29:A48"/>
     <mergeCell ref="F29:F34"/>
     <mergeCell ref="B35:H35"/>
-    <mergeCell ref="F7:F12"/>
-    <mergeCell ref="A7:A26"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="F36:F41"/>
     <mergeCell ref="B42:H42"/>
-    <mergeCell ref="F43:F48"/>
     <mergeCell ref="A49:H49"/>
     <mergeCell ref="B50:H50"/>
     <mergeCell ref="A51:A70"/>
@@ -33145,7 +33166,6 @@
     <mergeCell ref="F73:F78"/>
     <mergeCell ref="B79:H79"/>
     <mergeCell ref="B86:H86"/>
-    <mergeCell ref="A29:A48"/>
   </mergeCells>
   <conditionalFormatting sqref="F30:F34">
     <cfRule type="notContainsBlanks" dxfId="0" priority="1">
@@ -33166,7 +33186,7 @@
   </conditionalFormatting>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E7:E12 E14:E19 E21:E26 E29:E34 E36:E41 E43:E48 E51:E56 E58:E63 E65:E70 E73:E78 E80:E85 E87:E92 E95:E100 E102:E107 E109:E114 E117:E122 E124:E129 E131:E136 E139:E144 E146:E151 E153:E158 E161:E166 E168:E173 E175:E180">
-      <formula1>"To evaluate,0,0,33,0,66,1"</formula1>
+      <formula1>"To evaluate,0,1,2,3"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions/>

</xml_diff>